<commit_message>
Add row in demo tables
</commit_message>
<xml_diff>
--- a/Demo/Input/MRP_Drug_DrugGroup/Drug_DrugGroup_250314.xlsx
+++ b/Demo/Input/MRP_Drug_DrugGroup/Drug_DrugGroup_250314.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
   <si>
     <t xml:space="preserve">Drug-DrugGroup</t>
   </si>
@@ -119,6 +119,27 @@
   </si>
   <si>
     <t xml:space="preserve">Name des zweiten ATC Codes, wenn Kombipräparat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALDOXAN® 25 mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gleichzeitige Anwendung von starken CYP1A2-Inhibitoren (siehe Abschnitt 4.5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agomelatin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N06AX22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CYP1A2-Inhibitoren, stark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J01MA02 N06AB08 </t>
   </si>
 </sst>
 </file>
@@ -302,103 +323,103 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -687,7 +708,7 @@
   <dimension ref="A1:N1024"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="4" style="1" width="20.37"/>
@@ -892,20 +913,36 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>45413</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>35</v>
+      </c>
       <c r="F25" s="11"/>
       <c r="G25" s="11"/>
       <c r="H25" s="11"/>
       <c r="I25" s="11"/>
       <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="13"/>
+      <c r="K25" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11"/>
@@ -1055,7 +1092,7 @@
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
       <c r="L35" s="11"/>
-      <c r="M35" s="14"/>
+      <c r="M35" s="13"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11"/>
@@ -1100,7 +1137,7 @@
       <c r="J38" s="11"/>
       <c r="K38" s="11"/>
       <c r="L38" s="11"/>
-      <c r="M38" s="13"/>
+      <c r="M38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="11"/>
@@ -2119,7 +2156,7 @@
       <c r="J106" s="11"/>
       <c r="K106" s="11"/>
       <c r="L106" s="11"/>
-      <c r="M106" s="13"/>
+      <c r="M106" s="14"/>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="11"/>
@@ -2164,7 +2201,7 @@
       <c r="J109" s="11"/>
       <c r="K109" s="11"/>
       <c r="L109" s="11"/>
-      <c r="M109" s="13"/>
+      <c r="M109" s="14"/>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="11"/>
@@ -2373,7 +2410,7 @@
       <c r="J123" s="11"/>
       <c r="K123" s="11"/>
       <c r="L123" s="11"/>
-      <c r="M123" s="13"/>
+      <c r="M123" s="14"/>
     </row>
     <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="11"/>
@@ -4380,7 +4417,7 @@
       <c r="J257" s="11"/>
       <c r="K257" s="11"/>
       <c r="L257" s="11"/>
-      <c r="M257" s="13"/>
+      <c r="M257" s="14"/>
     </row>
     <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="11"/>
@@ -5640,7 +5677,7 @@
       <c r="J341" s="11"/>
       <c r="K341" s="11"/>
       <c r="L341" s="11"/>
-      <c r="M341" s="13"/>
+      <c r="M341" s="14"/>
     </row>
     <row r="342" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="11"/>
@@ -6645,7 +6682,7 @@
       <c r="J408" s="11"/>
       <c r="K408" s="11"/>
       <c r="L408" s="11"/>
-      <c r="M408" s="13"/>
+      <c r="M408" s="14"/>
     </row>
     <row r="409" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A409" s="11"/>
@@ -8010,7 +8047,7 @@
       <c r="J499" s="11"/>
       <c r="K499" s="11"/>
       <c r="L499" s="11"/>
-      <c r="M499" s="13"/>
+      <c r="M499" s="14"/>
     </row>
     <row r="500" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A500" s="11"/>
@@ -9015,7 +9052,7 @@
       <c r="J566" s="11"/>
       <c r="K566" s="11"/>
       <c r="L566" s="11"/>
-      <c r="M566" s="13"/>
+      <c r="M566" s="14"/>
     </row>
     <row r="567" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A567" s="11"/>
@@ -11825,7 +11862,7 @@
       <c r="J756" s="11"/>
       <c r="K756" s="11"/>
       <c r="L756" s="11"/>
-      <c r="M756" s="13"/>
+      <c r="M756" s="14"/>
     </row>
     <row r="757" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A757" s="11"/>
@@ -14149,7 +14186,7 @@
       <c r="J912" s="11"/>
       <c r="K912" s="11"/>
       <c r="L912" s="11"/>
-      <c r="M912" s="13"/>
+      <c r="M912" s="14"/>
     </row>
     <row r="913" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A913" s="11"/>
@@ -14194,7 +14231,7 @@
       <c r="J915" s="11"/>
       <c r="K915" s="11"/>
       <c r="L915" s="11"/>
-      <c r="M915" s="13"/>
+      <c r="M915" s="14"/>
     </row>
     <row r="916" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A916" s="11"/>

</xml_diff>